<commit_message>
Updated templates for new notification
</commit_message>
<xml_diff>
--- a/mosip_master/xlsx/template.xlsx
+++ b/mosip_master/xlsx/template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nira-registration\mosip-data\mosip_master\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TF-NIRA-REPOS\mosip-data\mosip_master\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8684C12B-95B2-42BA-AC14-985B73E3E5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F8B3F62-A12F-4FA4-B958-1BFB33170FCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3388" uniqueCount="955">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3415" uniqueCount="963">
   <si>
     <t>id</t>
   </si>
@@ -7506,6 +7506,33 @@
 &lt;/body&gt;
 &lt;/html&gt;</t>
   </si>
+  <si>
+    <t>Template for technical issue with error Email</t>
+  </si>
+  <si>
+    <t>Template for technical issue with error Subject</t>
+  </si>
+  <si>
+    <t>Template for technical issue with error SMS</t>
+  </si>
+  <si>
+    <t>RPR_TEC_ISSUE_ERROR_EMAIL</t>
+  </si>
+  <si>
+    <t>RPR_TEC_ISSUE_ERROR_EMAIL_SUB</t>
+  </si>
+  <si>
+    <t>RPR_TEC_ISSUE_ERROR_SMS</t>
+  </si>
+  <si>
+    <t>Dear $!surname_eng $!givenName_eng,
+	We regret to inform you that your request for a National Identification Number (NIN) $!MASKEDNIN linked to Registration ID $!RID has encountered an issue - $!FAILURE_REASON.
+	Please restart the registration process by submitting a new application.
+	Thank you for your understanding.</t>
+  </si>
+  <si>
+    <t>Application failed</t>
+  </si>
 </sst>
 </file>
 
@@ -20971,6 +20998,111 @@
         <v>911</v>
       </c>
     </row>
+    <row r="375" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+      <c r="A375">
+        <v>2007</v>
+      </c>
+      <c r="B375" t="s">
+        <v>955</v>
+      </c>
+      <c r="C375" t="s">
+        <v>955</v>
+      </c>
+      <c r="D375" t="s">
+        <v>12</v>
+      </c>
+      <c r="E375" t="s">
+        <v>13</v>
+      </c>
+      <c r="F375" s="4" t="s">
+        <v>961</v>
+      </c>
+      <c r="G375">
+        <v>10003</v>
+      </c>
+      <c r="H375" t="s">
+        <v>31</v>
+      </c>
+      <c r="I375" t="s">
+        <v>958</v>
+      </c>
+      <c r="J375" t="s">
+        <v>17</v>
+      </c>
+      <c r="K375" t="s">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="376" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A376">
+        <v>2008</v>
+      </c>
+      <c r="B376" t="s">
+        <v>956</v>
+      </c>
+      <c r="C376" t="s">
+        <v>956</v>
+      </c>
+      <c r="D376" t="s">
+        <v>12</v>
+      </c>
+      <c r="E376" t="s">
+        <v>13</v>
+      </c>
+      <c r="F376" s="4" t="s">
+        <v>962</v>
+      </c>
+      <c r="G376">
+        <v>10003</v>
+      </c>
+      <c r="H376" t="s">
+        <v>31</v>
+      </c>
+      <c r="I376" t="s">
+        <v>959</v>
+      </c>
+      <c r="J376" t="s">
+        <v>17</v>
+      </c>
+      <c r="K376" t="s">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="377" spans="1:11" ht="165" x14ac:dyDescent="0.25">
+      <c r="A377">
+        <v>2009</v>
+      </c>
+      <c r="B377" t="s">
+        <v>957</v>
+      </c>
+      <c r="C377" t="s">
+        <v>957</v>
+      </c>
+      <c r="D377" t="s">
+        <v>12</v>
+      </c>
+      <c r="E377" t="s">
+        <v>13</v>
+      </c>
+      <c r="F377" s="4" t="s">
+        <v>961</v>
+      </c>
+      <c r="G377">
+        <v>10003</v>
+      </c>
+      <c r="H377" t="s">
+        <v>31</v>
+      </c>
+      <c r="I377" t="s">
+        <v>960</v>
+      </c>
+      <c r="J377" t="s">
+        <v>17</v>
+      </c>
+      <c r="K377" t="s">
+        <v>911</v>
+      </c>
+    </row>
     <row r="622" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F622" s="1"/>
     </row>

</xml_diff>